<commit_message>
Ship Complete-Cable MVP backend: rules v2, library governance, and full BOM.
Adds ruleset-gated validation, starter catalog seeding, library-resolved BOM lines (including accessories), optimistic snapshot concurrency, observability, and export reliability needed for one cable end to end.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/wirelist-template.xlsx
+++ b/data/wirelist-template.xlsx
@@ -33,7 +33,7 @@
     <definedName name="NO">#REF!</definedName>
     <definedName name="ORIGINATOR">#REF!</definedName>
     <definedName name="PN">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Wirelist!$A$1:$O$151</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Wirelist!$A$1:$P$151</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Wirelist!$1:$1</definedName>
     <definedName name="STATUS">#REF!</definedName>
     <definedName name="YES">#REF!</definedName>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Run #</t>
   </si>
@@ -83,6 +83,9 @@
   </si>
   <si>
     <t>Length (in)</t>
+  </si>
+  <si>
+    <t>Sleeving</t>
   </si>
   <si>
     <t>Wire Color</t>
@@ -1568,7 +1571,7 @@
     <tabColor rgb="FF00B050"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O151"/>
+  <dimension ref="A1:P151"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" style="11" customWidth="1"/>
@@ -1589,7 +1592,7 @@
     <col min="16" max="16" width="3.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="3" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="3" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1635,8 +1638,11 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1647,15 +1653,16 @@
       <c r="F2" s="7"/>
       <c r="G2" s="8"/>
       <c r="H2" s="5"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="8"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="4"/>
       <c r="N2" s="8"/>
-      <c r="O2" s="9"/>
-    </row>
-    <row r="3" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O2" s="8"/>
+      <c r="P2" s="9"/>
+    </row>
+    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1674,7 +1681,7 @@
       <c r="N3" s="8"/>
       <c r="O3" s="10"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1693,7 +1700,7 @@
       <c r="N4" s="8"/>
       <c r="O4" s="10"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1712,7 +1719,7 @@
       <c r="N5" s="8"/>
       <c r="O5" s="10"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -1731,7 +1738,7 @@
       <c r="N6" s="8"/>
       <c r="O6" s="10"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -1750,7 +1757,7 @@
       <c r="N7" s="8"/>
       <c r="O7" s="10"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -1769,7 +1776,7 @@
       <c r="N8" s="8"/>
       <c r="O8" s="10"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -1788,7 +1795,7 @@
       <c r="N9" s="8"/>
       <c r="O9" s="10"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -1807,7 +1814,7 @@
       <c r="N10" s="8"/>
       <c r="O10" s="10"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -1826,7 +1833,7 @@
       <c r="N11" s="8"/>
       <c r="O11" s="10"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -1845,7 +1852,7 @@
       <c r="N12" s="8"/>
       <c r="O12" s="10"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -1864,7 +1871,7 @@
       <c r="N13" s="8"/>
       <c r="O13" s="10"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -1883,7 +1890,7 @@
       <c r="N14" s="8"/>
       <c r="O14" s="10"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -1902,7 +1909,7 @@
       <c r="N15" s="8"/>
       <c r="O15" s="10"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -1921,7 +1928,7 @@
       <c r="N16" s="8"/>
       <c r="O16" s="10"/>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -1940,7 +1947,7 @@
       <c r="N17" s="8"/>
       <c r="O17" s="10"/>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>17</v>
       </c>
@@ -1959,7 +1966,7 @@
       <c r="N18" s="8"/>
       <c r="O18" s="10"/>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>18</v>
       </c>
@@ -1978,7 +1985,7 @@
       <c r="N19" s="8"/>
       <c r="O19" s="10"/>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>19</v>
       </c>
@@ -1997,7 +2004,7 @@
       <c r="N20" s="8"/>
       <c r="O20" s="10"/>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <v>20</v>
       </c>
@@ -2016,7 +2023,7 @@
       <c r="N21" s="8"/>
       <c r="O21" s="10"/>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>21</v>
       </c>
@@ -2035,7 +2042,7 @@
       <c r="N22" s="8"/>
       <c r="O22" s="10"/>
     </row>
-    <row r="23" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>22</v>
       </c>
@@ -2054,7 +2061,7 @@
       <c r="N23" s="8"/>
       <c r="O23" s="10"/>
     </row>
-    <row r="24" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <v>23</v>
       </c>
@@ -2073,7 +2080,7 @@
       <c r="N24" s="8"/>
       <c r="O24" s="10"/>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <v>24</v>
       </c>
@@ -2092,7 +2099,7 @@
       <c r="N25" s="8"/>
       <c r="O25" s="10"/>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>25</v>
       </c>
@@ -2110,7 +2117,7 @@
       <c r="N26" s="8"/>
       <c r="O26" s="10"/>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>26</v>
       </c>
@@ -2128,7 +2135,7 @@
       <c r="N27" s="8"/>
       <c r="O27" s="10"/>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
         <v>27</v>
       </c>
@@ -2146,7 +2153,7 @@
       <c r="N28" s="8"/>
       <c r="O28" s="10"/>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <v>28</v>
       </c>
@@ -2164,7 +2171,7 @@
       <c r="N29" s="8"/>
       <c r="O29" s="10"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -2182,7 +2189,7 @@
       <c r="N30" s="8"/>
       <c r="O30" s="10"/>
     </row>
-    <row r="31" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <v>30</v>
       </c>
@@ -2201,7 +2208,7 @@
       <c r="N31" s="8"/>
       <c r="O31" s="10"/>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <v>31</v>
       </c>
@@ -2220,7 +2227,7 @@
       <c r="N32" s="8"/>
       <c r="O32" s="10"/>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
         <v>32</v>
       </c>
@@ -2239,7 +2246,7 @@
       <c r="N33" s="8"/>
       <c r="O33" s="10"/>
     </row>
-    <row r="34" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
         <v>33</v>
       </c>
@@ -2258,7 +2265,7 @@
       <c r="N34" s="8"/>
       <c r="O34" s="10"/>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="4">
         <v>34</v>
       </c>
@@ -2277,7 +2284,7 @@
       <c r="N35" s="8"/>
       <c r="O35" s="10"/>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
         <v>35</v>
       </c>
@@ -2296,7 +2303,7 @@
       <c r="N36" s="8"/>
       <c r="O36" s="10"/>
     </row>
-    <row r="37" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4">
         <v>36</v>
       </c>
@@ -2315,7 +2322,7 @@
       <c r="N37" s="8"/>
       <c r="O37" s="10"/>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="4">
         <v>37</v>
       </c>
@@ -2334,7 +2341,7 @@
       <c r="N38" s="8"/>
       <c r="O38" s="10"/>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="4">
         <v>38</v>
       </c>
@@ -2353,7 +2360,7 @@
       <c r="N39" s="8"/>
       <c r="O39" s="10"/>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="4">
         <v>39</v>
       </c>
@@ -2372,7 +2379,7 @@
       <c r="N40" s="8"/>
       <c r="O40" s="10"/>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="4">
         <v>40</v>
       </c>
@@ -2391,7 +2398,7 @@
       <c r="N41" s="8"/>
       <c r="O41" s="10"/>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="4">
         <v>41</v>
       </c>
@@ -2410,7 +2417,7 @@
       <c r="N42" s="8"/>
       <c r="O42" s="10"/>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" s="4">
         <v>42</v>
       </c>
@@ -2429,7 +2436,7 @@
       <c r="N43" s="8"/>
       <c r="O43" s="10"/>
     </row>
-    <row r="44" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="4">
         <v>43</v>
       </c>
@@ -2448,7 +2455,7 @@
       <c r="N44" s="8"/>
       <c r="O44" s="10"/>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="4">
         <v>44</v>
       </c>
@@ -2467,7 +2474,7 @@
       <c r="N45" s="8"/>
       <c r="O45" s="10"/>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="4">
         <v>45</v>
       </c>
@@ -2486,7 +2493,7 @@
       <c r="N46" s="8"/>
       <c r="O46" s="10"/>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" s="4">
         <v>46</v>
       </c>
@@ -2505,7 +2512,7 @@
       <c r="N47" s="8"/>
       <c r="O47" s="10"/>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="4">
         <v>47</v>
       </c>
@@ -2524,7 +2531,7 @@
       <c r="N48" s="8"/>
       <c r="O48" s="10"/>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="4">
         <v>48</v>
       </c>
@@ -2543,7 +2550,7 @@
       <c r="N49" s="14"/>
       <c r="O49" s="10"/>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="4">
         <v>49</v>
       </c>
@@ -2562,7 +2569,7 @@
       <c r="N50" s="14"/>
       <c r="O50" s="10"/>
     </row>
-    <row r="51" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="4">
         <v>50</v>
       </c>
@@ -2581,7 +2588,7 @@
       <c r="N51" s="14"/>
       <c r="O51" s="10"/>
     </row>
-    <row r="52" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="4">
         <v>51</v>
       </c>
@@ -2600,7 +2607,7 @@
       <c r="N52" s="14"/>
       <c r="O52" s="10"/>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="4">
         <v>52</v>
       </c>
@@ -2619,7 +2626,7 @@
       <c r="N53" s="14"/>
       <c r="O53" s="10"/>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="4">
         <v>53</v>
       </c>
@@ -2638,7 +2645,7 @@
       <c r="N54" s="14"/>
       <c r="O54" s="10"/>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="4">
         <v>54</v>
       </c>
@@ -2657,7 +2664,7 @@
       <c r="N55" s="14"/>
       <c r="O55" s="10"/>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="4">
         <v>55</v>
       </c>
@@ -2676,7 +2683,7 @@
       <c r="N56" s="14"/>
       <c r="O56" s="10"/>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" s="4">
         <v>56</v>
       </c>
@@ -2695,7 +2702,7 @@
       <c r="N57" s="14"/>
       <c r="O57" s="10"/>
     </row>
-    <row r="58" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="4">
         <v>57</v>
       </c>
@@ -2714,7 +2721,7 @@
       <c r="N58" s="14"/>
       <c r="O58" s="10"/>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="4">
         <v>58</v>
       </c>
@@ -2733,7 +2740,7 @@
       <c r="N59" s="14"/>
       <c r="O59" s="10"/>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="4">
         <v>59</v>
       </c>
@@ -2752,7 +2759,7 @@
       <c r="N60" s="14"/>
       <c r="O60" s="10"/>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" s="4">
         <v>60</v>
       </c>
@@ -2771,7 +2778,7 @@
       <c r="N61" s="14"/>
       <c r="O61" s="10"/>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="4">
         <v>61</v>
       </c>
@@ -2790,7 +2797,7 @@
       <c r="N62" s="14"/>
       <c r="O62" s="10"/>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="4">
         <v>62</v>
       </c>
@@ -2809,7 +2816,7 @@
       <c r="N63" s="14"/>
       <c r="O63" s="10"/>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" s="4">
         <v>63</v>
       </c>
@@ -2828,7 +2835,7 @@
       <c r="N64" s="14"/>
       <c r="O64" s="10"/>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="4">
         <v>64</v>
       </c>
@@ -2847,7 +2854,7 @@
       <c r="N65" s="14"/>
       <c r="O65" s="10"/>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="4">
         <v>65</v>
       </c>
@@ -2866,7 +2873,7 @@
       <c r="N66" s="14"/>
       <c r="O66" s="10"/>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="4">
         <v>66</v>
       </c>
@@ -2885,7 +2892,7 @@
       <c r="N67" s="14"/>
       <c r="O67" s="10"/>
     </row>
-    <row r="68" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
         <v>67</v>
       </c>
@@ -2904,7 +2911,7 @@
       <c r="N68" s="14"/>
       <c r="O68" s="10"/>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="4">
         <v>68</v>
       </c>
@@ -2923,7 +2930,7 @@
       <c r="N69" s="14"/>
       <c r="O69" s="10"/>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
         <v>69</v>
       </c>
@@ -2942,7 +2949,7 @@
       <c r="N70" s="14"/>
       <c r="O70" s="10"/>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="4">
         <v>70</v>
       </c>
@@ -2961,7 +2968,7 @@
       <c r="N71" s="14"/>
       <c r="O71" s="10"/>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="4">
         <v>71</v>
       </c>
@@ -2980,7 +2987,7 @@
       <c r="N72" s="14"/>
       <c r="O72" s="10"/>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="4">
         <v>72</v>
       </c>
@@ -2999,7 +3006,7 @@
       <c r="N73" s="14"/>
       <c r="O73" s="10"/>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="4">
         <v>73</v>
       </c>
@@ -3018,7 +3025,7 @@
       <c r="N74" s="14"/>
       <c r="O74" s="10"/>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="4">
         <v>74</v>
       </c>
@@ -3037,7 +3044,7 @@
       <c r="N75" s="14"/>
       <c r="O75" s="10"/>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="4">
         <v>75</v>
       </c>
@@ -3056,7 +3063,7 @@
       <c r="N76" s="14"/>
       <c r="O76" s="10"/>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="4">
         <v>76</v>
       </c>
@@ -3075,7 +3082,7 @@
       <c r="N77" s="14"/>
       <c r="O77" s="10"/>
     </row>
-    <row r="78" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="4">
         <v>77</v>
       </c>
@@ -3094,7 +3101,7 @@
       <c r="N78" s="14"/>
       <c r="O78" s="10"/>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="4">
         <v>78</v>
       </c>
@@ -3113,7 +3120,7 @@
       <c r="N79" s="14"/>
       <c r="O79" s="10"/>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
         <v>79</v>
       </c>
@@ -3132,7 +3139,7 @@
       <c r="N80" s="14"/>
       <c r="O80" s="10"/>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="4">
         <v>80</v>
       </c>
@@ -3151,7 +3158,7 @@
       <c r="N81" s="14"/>
       <c r="O81" s="10"/>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
         <v>81</v>
       </c>
@@ -3170,7 +3177,7 @@
       <c r="N82" s="14"/>
       <c r="O82" s="10"/>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="4">
         <v>82</v>
       </c>
@@ -3189,7 +3196,7 @@
       <c r="N83" s="14"/>
       <c r="O83" s="10"/>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
         <v>83</v>
       </c>
@@ -3208,7 +3215,7 @@
       <c r="N84" s="14"/>
       <c r="O84" s="10"/>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="4">
         <v>84</v>
       </c>
@@ -3227,7 +3234,7 @@
       <c r="N85" s="14"/>
       <c r="O85" s="10"/>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="4">
         <v>85</v>
       </c>
@@ -3246,7 +3253,7 @@
       <c r="N86" s="14"/>
       <c r="O86" s="10"/>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="4">
         <v>86</v>
       </c>
@@ -3265,7 +3272,7 @@
       <c r="N87" s="14"/>
       <c r="O87" s="10"/>
     </row>
-    <row r="88" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="4">
         <v>87</v>
       </c>
@@ -3284,7 +3291,7 @@
       <c r="N88" s="14"/>
       <c r="O88" s="10"/>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" s="4">
         <v>88</v>
       </c>
@@ -3303,7 +3310,7 @@
       <c r="N89" s="14"/>
       <c r="O89" s="10"/>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="4">
         <v>89</v>
       </c>
@@ -3322,7 +3329,7 @@
       <c r="N90" s="14"/>
       <c r="O90" s="10"/>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" s="4">
         <v>90</v>
       </c>
@@ -3341,7 +3348,7 @@
       <c r="N91" s="14"/>
       <c r="O91" s="10"/>
     </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" s="4">
         <v>91</v>
       </c>
@@ -3360,7 +3367,7 @@
       <c r="N92" s="14"/>
       <c r="O92" s="10"/>
     </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" s="4">
         <v>92</v>
       </c>
@@ -3379,7 +3386,7 @@
       <c r="N93" s="14"/>
       <c r="O93" s="10"/>
     </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="4">
         <v>93</v>
       </c>
@@ -3398,7 +3405,7 @@
       <c r="N94" s="14"/>
       <c r="O94" s="10"/>
     </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95" s="4">
         <v>94</v>
       </c>
@@ -3417,7 +3424,7 @@
       <c r="N95" s="14"/>
       <c r="O95" s="10"/>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" s="4">
         <v>95</v>
       </c>
@@ -3436,7 +3443,7 @@
       <c r="N96" s="14"/>
       <c r="O96" s="10"/>
     </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A97" s="4">
         <v>96</v>
       </c>
@@ -3455,7 +3462,7 @@
       <c r="N97" s="14"/>
       <c r="O97" s="10"/>
     </row>
-    <row r="98" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="4">
         <v>97</v>
       </c>
@@ -3474,7 +3481,7 @@
       <c r="N98" s="14"/>
       <c r="O98" s="10"/>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A99" s="4">
         <v>98</v>
       </c>
@@ -3493,7 +3500,7 @@
       <c r="N99" s="14"/>
       <c r="O99" s="10"/>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
         <v>99</v>
       </c>
@@ -3512,7 +3519,7 @@
       <c r="N100" s="14"/>
       <c r="O100" s="10"/>
     </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
         <v>100</v>
       </c>
@@ -3531,7 +3538,7 @@
       <c r="N101" s="14"/>
       <c r="O101" s="10"/>
     </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
         <v>101</v>
       </c>
@@ -3550,7 +3557,7 @@
       <c r="N102" s="14"/>
       <c r="O102" s="10"/>
     </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
         <v>102</v>
       </c>
@@ -3569,7 +3576,7 @@
       <c r="N103" s="14"/>
       <c r="O103" s="10"/>
     </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
         <v>103</v>
       </c>
@@ -3588,7 +3595,7 @@
       <c r="N104" s="14"/>
       <c r="O104" s="10"/>
     </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
         <v>104</v>
       </c>
@@ -3607,7 +3614,7 @@
       <c r="N105" s="14"/>
       <c r="O105" s="10"/>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A106" s="4">
         <v>105</v>
       </c>
@@ -3626,7 +3633,7 @@
       <c r="N106" s="14"/>
       <c r="O106" s="10"/>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
         <v>106</v>
       </c>
@@ -3645,7 +3652,7 @@
       <c r="N107" s="14"/>
       <c r="O107" s="10"/>
     </row>
-    <row r="108" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
         <v>107</v>
       </c>
@@ -3664,7 +3671,7 @@
       <c r="N108" s="14"/>
       <c r="O108" s="10"/>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
         <v>108</v>
       </c>
@@ -3683,7 +3690,7 @@
       <c r="N109" s="14"/>
       <c r="O109" s="10"/>
     </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
         <v>109</v>
       </c>
@@ -3702,7 +3709,7 @@
       <c r="N110" s="14"/>
       <c r="O110" s="10"/>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
         <v>110</v>
       </c>
@@ -3721,7 +3728,7 @@
       <c r="N111" s="14"/>
       <c r="O111" s="10"/>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
         <v>111</v>
       </c>
@@ -3740,7 +3747,7 @@
       <c r="N112" s="14"/>
       <c r="O112" s="10"/>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A113" s="4">
         <v>112</v>
       </c>
@@ -3759,7 +3766,7 @@
       <c r="N113" s="14"/>
       <c r="O113" s="10"/>
     </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A114" s="4">
         <v>113</v>
       </c>
@@ -3778,7 +3785,7 @@
       <c r="N114" s="14"/>
       <c r="O114" s="10"/>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A115" s="4">
         <v>114</v>
       </c>
@@ -3797,7 +3804,7 @@
       <c r="N115" s="14"/>
       <c r="O115" s="10"/>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A116" s="4">
         <v>115</v>
       </c>
@@ -3816,7 +3823,7 @@
       <c r="N116" s="14"/>
       <c r="O116" s="10"/>
     </row>
-    <row r="117" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="4">
         <v>116</v>
       </c>
@@ -3835,7 +3842,7 @@
       <c r="N117" s="14"/>
       <c r="O117" s="10"/>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A118" s="4">
         <v>117</v>
       </c>
@@ -3854,7 +3861,7 @@
       <c r="N118" s="14"/>
       <c r="O118" s="10"/>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A119" s="4">
         <v>118</v>
       </c>
@@ -3873,7 +3880,7 @@
       <c r="N119" s="14"/>
       <c r="O119" s="10"/>
     </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A120" s="4">
         <v>119</v>
       </c>
@@ -3892,7 +3899,7 @@
       <c r="N120" s="14"/>
       <c r="O120" s="10"/>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A121" s="4">
         <v>120</v>
       </c>
@@ -3911,7 +3918,7 @@
       <c r="N121" s="14"/>
       <c r="O121" s="10"/>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A122" s="4">
         <v>121</v>
       </c>
@@ -3930,7 +3937,7 @@
       <c r="N122" s="14"/>
       <c r="O122" s="10"/>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A123" s="4">
         <v>122</v>
       </c>
@@ -3949,7 +3956,7 @@
       <c r="N123" s="14"/>
       <c r="O123" s="10"/>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
         <v>123</v>
       </c>
@@ -3968,7 +3975,7 @@
       <c r="N124" s="14"/>
       <c r="O124" s="10"/>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
         <v>124</v>
       </c>
@@ -3987,7 +3994,7 @@
       <c r="N125" s="14"/>
       <c r="O125" s="10"/>
     </row>
-    <row r="126" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
         <v>125</v>
       </c>
@@ -4006,7 +4013,7 @@
       <c r="N126" s="14"/>
       <c r="O126" s="10"/>
     </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A127" s="4">
         <v>126</v>
       </c>
@@ -4025,145 +4032,145 @@
       <c r="N127" s="16"/>
       <c r="O127" s="18"/>
     </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A128" s="4">
         <v>127</v>
       </c>
       <c r="O128" s="20"/>
     </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A129" s="4">
         <v>128</v>
       </c>
       <c r="O129" s="20"/>
     </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A130" s="4">
         <v>129</v>
       </c>
       <c r="O130" s="20"/>
     </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A131" s="4">
         <v>130</v>
       </c>
       <c r="O131" s="20"/>
     </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A132" s="4">
         <v>131</v>
       </c>
       <c r="O132" s="20"/>
     </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A133" s="4">
         <v>132</v>
       </c>
       <c r="O133" s="20"/>
     </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A134" s="4">
         <v>133</v>
       </c>
       <c r="O134" s="20"/>
     </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A135" s="4">
         <v>134</v>
       </c>
       <c r="O135" s="20"/>
     </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A136" s="4">
         <v>135</v>
       </c>
       <c r="O136" s="20"/>
     </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A137" s="4">
         <v>136</v>
       </c>
       <c r="O137" s="20"/>
     </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A138" s="4">
         <v>137</v>
       </c>
       <c r="O138" s="20"/>
     </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A139" s="4">
         <v>138</v>
       </c>
       <c r="O139" s="20"/>
     </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A140" s="4">
         <v>139</v>
       </c>
       <c r="O140" s="20"/>
     </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A141" s="4">
         <v>140</v>
       </c>
       <c r="O141" s="20"/>
     </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A142" s="4">
         <v>141</v>
       </c>
       <c r="O142" s="20"/>
     </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A143" s="4">
         <v>142</v>
       </c>
       <c r="O143" s="20"/>
     </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A144" s="4">
         <v>143</v>
       </c>
       <c r="O144" s="20"/>
     </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A145" s="4">
         <v>144</v>
       </c>
       <c r="O145" s="20"/>
     </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A146" s="4">
         <v>145</v>
       </c>
       <c r="O146" s="20"/>
     </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A147" s="4">
         <v>146</v>
       </c>
       <c r="O147" s="20"/>
     </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A148" s="4">
         <v>147</v>
       </c>
       <c r="O148" s="20"/>
     </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A149" s="4">
         <v>148</v>
       </c>
       <c r="O149" s="20"/>
     </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A150" s="4">
         <v>149</v>
       </c>
       <c r="O150" s="20"/>
     </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A151" s="4">
         <v>150</v>
       </c>

</xml_diff>

<commit_message>
Ship the parts-model item database, CPQ import, and Vercel Production/Test hosting.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/wirelist-template.xlsx
+++ b/data/wirelist-template.xlsx
@@ -33,7 +33,7 @@
     <definedName name="NO">#REF!</definedName>
     <definedName name="ORIGINATOR">#REF!</definedName>
     <definedName name="PN">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Wirelist!$A$1:$P$151</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Wirelist!$A$1:$O$151</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Wirelist!$1:$1</definedName>
     <definedName name="STATUS">#REF!</definedName>
     <definedName name="YES">#REF!</definedName>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Run #</t>
   </si>
@@ -83,9 +83,6 @@
   </si>
   <si>
     <t>Length (in)</t>
-  </si>
-  <si>
-    <t>Sleeving</t>
   </si>
   <si>
     <t>Wire Color</t>
@@ -1571,7 +1568,7 @@
     <tabColor rgb="FF00B050"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P151"/>
+  <dimension ref="A1:O151"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" style="11" customWidth="1"/>
@@ -1581,18 +1578,17 @@
     <col min="5" max="5" width="8.42578125" style="11" customWidth="1"/>
     <col min="6" max="6" width="22.7109375" style="19" customWidth="1"/>
     <col min="7" max="7" width="9.85546875" style="11" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" style="11" customWidth="1"/>
-    <col min="9" max="9" width="7.140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.140625" style="11" customWidth="1"/>
-    <col min="11" max="11" width="12" style="19" customWidth="1"/>
-    <col min="12" max="12" width="15.5703125" style="11" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.5703125" style="11" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10" style="11" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="41.140625" style="11" customWidth="1"/>
-    <col min="16" max="16" width="3.5703125" customWidth="1"/>
+    <col min="8" max="8" width="7.140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" style="11" customWidth="1"/>
+    <col min="10" max="10" width="12" style="19" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" style="11" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.5703125" style="11" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10" style="11" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="41.140625" style="11" customWidth="1"/>
+    <col min="15" max="15" width="3.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="3" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="3" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1620,10 +1616,10 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
@@ -1638,11 +1634,8 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1653,16 +1646,15 @@
       <c r="F2" s="7"/>
       <c r="G2" s="8"/>
       <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="4"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="8"/>
       <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="9"/>
-    </row>
-    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O2" s="9"/>
+    </row>
+    <row r="3" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1672,16 +1664,15 @@
       <c r="E3" s="5"/>
       <c r="F3" s="7"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="4"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="8"/>
       <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="10"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N3" s="10"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1691,16 +1682,15 @@
       <c r="E4" s="5"/>
       <c r="F4" s="7"/>
       <c r="G4" s="8"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="4"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="8"/>
       <c r="M4" s="8"/>
-      <c r="N4" s="8"/>
-      <c r="O4" s="10"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N4" s="10"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1710,16 +1700,15 @@
       <c r="E5" s="5"/>
       <c r="F5" s="7"/>
       <c r="G5" s="8"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="4"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="8"/>
       <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="10"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N5" s="10"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -1729,16 +1718,15 @@
       <c r="E6" s="5"/>
       <c r="F6" s="7"/>
       <c r="G6" s="8"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="4"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="8"/>
       <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="10"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N6" s="10"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -1748,16 +1736,15 @@
       <c r="E7" s="5"/>
       <c r="F7" s="7"/>
       <c r="G7" s="8"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="4"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="8"/>
       <c r="M7" s="8"/>
-      <c r="N7" s="8"/>
-      <c r="O7" s="10"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N7" s="10"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -1767,16 +1754,15 @@
       <c r="E8" s="5"/>
       <c r="F8" s="7"/>
       <c r="G8" s="8"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="4"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="8"/>
       <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="10"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N8" s="10"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -1786,16 +1772,15 @@
       <c r="E9" s="5"/>
       <c r="F9" s="7"/>
       <c r="G9" s="8"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="4"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="8"/>
       <c r="M9" s="8"/>
-      <c r="N9" s="8"/>
-      <c r="O9" s="10"/>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N9" s="10"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -1805,16 +1790,15 @@
       <c r="E10" s="5"/>
       <c r="F10" s="7"/>
       <c r="G10" s="8"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="4"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="8"/>
       <c r="M10" s="8"/>
-      <c r="N10" s="8"/>
-      <c r="O10" s="10"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N10" s="10"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -1824,16 +1808,15 @@
       <c r="E11" s="5"/>
       <c r="F11" s="7"/>
       <c r="G11" s="8"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="4"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="8"/>
       <c r="M11" s="8"/>
-      <c r="N11" s="8"/>
-      <c r="O11" s="10"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N11" s="10"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -1843,16 +1826,15 @@
       <c r="E12" s="5"/>
       <c r="F12" s="7"/>
       <c r="G12" s="8"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="4"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="8"/>
       <c r="M12" s="8"/>
-      <c r="N12" s="8"/>
-      <c r="O12" s="10"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N12" s="10"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -1862,16 +1844,15 @@
       <c r="E13" s="5"/>
       <c r="F13" s="7"/>
       <c r="G13" s="8"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="4"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="8"/>
       <c r="M13" s="8"/>
-      <c r="N13" s="8"/>
-      <c r="O13" s="10"/>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N13" s="10"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -1881,16 +1862,15 @@
       <c r="E14" s="5"/>
       <c r="F14" s="7"/>
       <c r="G14" s="8"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="4"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="8"/>
       <c r="M14" s="8"/>
-      <c r="N14" s="8"/>
-      <c r="O14" s="10"/>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N14" s="10"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -1900,16 +1880,15 @@
       <c r="E15" s="5"/>
       <c r="F15" s="7"/>
       <c r="G15" s="8"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="4"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="8"/>
       <c r="M15" s="8"/>
-      <c r="N15" s="8"/>
-      <c r="O15" s="10"/>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N15" s="10"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -1919,16 +1898,15 @@
       <c r="E16" s="5"/>
       <c r="F16" s="7"/>
       <c r="G16" s="8"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="4"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="8"/>
       <c r="M16" s="8"/>
-      <c r="N16" s="8"/>
-      <c r="O16" s="10"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N16" s="10"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -1938,16 +1916,15 @@
       <c r="E17" s="5"/>
       <c r="F17" s="7"/>
       <c r="G17" s="8"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="4"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="8"/>
       <c r="M17" s="8"/>
-      <c r="N17" s="8"/>
-      <c r="O17" s="10"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N17" s="10"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>17</v>
       </c>
@@ -1957,16 +1934,15 @@
       <c r="E18" s="5"/>
       <c r="F18" s="7"/>
       <c r="G18" s="8"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="4"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="8"/>
       <c r="M18" s="8"/>
-      <c r="N18" s="8"/>
-      <c r="O18" s="10"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N18" s="10"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>18</v>
       </c>
@@ -1976,16 +1952,15 @@
       <c r="E19" s="5"/>
       <c r="F19" s="7"/>
       <c r="G19" s="8"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="4"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="8"/>
       <c r="M19" s="8"/>
-      <c r="N19" s="8"/>
-      <c r="O19" s="10"/>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N19" s="10"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>19</v>
       </c>
@@ -1995,16 +1970,15 @@
       <c r="E20" s="5"/>
       <c r="F20" s="7"/>
       <c r="G20" s="8"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="6"/>
-      <c r="L20" s="4"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="6"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="8"/>
       <c r="M20" s="8"/>
-      <c r="N20" s="8"/>
-      <c r="O20" s="10"/>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N20" s="10"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <v>20</v>
       </c>
@@ -2014,16 +1988,15 @@
       <c r="E21" s="5"/>
       <c r="F21" s="7"/>
       <c r="G21" s="8"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="4"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="8"/>
       <c r="M21" s="8"/>
-      <c r="N21" s="8"/>
-      <c r="O21" s="10"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N21" s="10"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>21</v>
       </c>
@@ -2033,16 +2006,15 @@
       <c r="E22" s="5"/>
       <c r="F22" s="7"/>
       <c r="G22" s="8"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="6"/>
-      <c r="L22" s="4"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="6"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="8"/>
       <c r="M22" s="8"/>
-      <c r="N22" s="8"/>
-      <c r="O22" s="10"/>
-    </row>
-    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N22" s="10"/>
+    </row>
+    <row r="23" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>22</v>
       </c>
@@ -2052,16 +2024,15 @@
       <c r="E23" s="5"/>
       <c r="F23" s="7"/>
       <c r="G23" s="8"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="6"/>
-      <c r="L23" s="4"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="8"/>
       <c r="M23" s="8"/>
-      <c r="N23" s="8"/>
-      <c r="O23" s="10"/>
-    </row>
-    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N23" s="10"/>
+    </row>
+    <row r="24" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <v>23</v>
       </c>
@@ -2071,16 +2042,15 @@
       <c r="E24" s="5"/>
       <c r="F24" s="7"/>
       <c r="G24" s="8"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="6"/>
-      <c r="L24" s="4"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="6"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="8"/>
       <c r="M24" s="8"/>
-      <c r="N24" s="8"/>
-      <c r="O24" s="10"/>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N24" s="10"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <v>24</v>
       </c>
@@ -2090,16 +2060,15 @@
       <c r="E25" s="5"/>
       <c r="F25" s="7"/>
       <c r="G25" s="8"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="6"/>
-      <c r="L25" s="4"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="8"/>
       <c r="M25" s="8"/>
-      <c r="N25" s="8"/>
-      <c r="O25" s="10"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N25" s="10"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>25</v>
       </c>
@@ -2108,16 +2077,15 @@
       <c r="D26" s="6"/>
       <c r="E26" s="5"/>
       <c r="F26" s="7"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="5"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="6"/>
       <c r="K26" s="6"/>
-      <c r="L26" s="6"/>
+      <c r="L26" s="8"/>
       <c r="M26" s="8"/>
-      <c r="N26" s="8"/>
-      <c r="O26" s="10"/>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N26" s="10"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>26</v>
       </c>
@@ -2126,16 +2094,15 @@
       <c r="D27" s="6"/>
       <c r="E27" s="5"/>
       <c r="F27" s="7"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="5"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="6"/>
       <c r="K27" s="6"/>
-      <c r="L27" s="6"/>
+      <c r="L27" s="8"/>
       <c r="M27" s="8"/>
-      <c r="N27" s="8"/>
-      <c r="O27" s="10"/>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N27" s="10"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
         <v>27</v>
       </c>
@@ -2144,16 +2111,15 @@
       <c r="D28" s="6"/>
       <c r="E28" s="5"/>
       <c r="F28" s="7"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="8"/>
-      <c r="J28" s="5"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="6"/>
       <c r="K28" s="6"/>
-      <c r="L28" s="6"/>
+      <c r="L28" s="8"/>
       <c r="M28" s="8"/>
-      <c r="N28" s="8"/>
-      <c r="O28" s="10"/>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N28" s="10"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <v>28</v>
       </c>
@@ -2162,16 +2128,15 @@
       <c r="D29" s="6"/>
       <c r="E29" s="5"/>
       <c r="F29" s="7"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="8"/>
-      <c r="J29" s="5"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="6"/>
       <c r="K29" s="6"/>
-      <c r="L29" s="6"/>
+      <c r="L29" s="8"/>
       <c r="M29" s="8"/>
-      <c r="N29" s="8"/>
-      <c r="O29" s="10"/>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N29" s="10"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -2180,16 +2145,15 @@
       <c r="D30" s="6"/>
       <c r="E30" s="5"/>
       <c r="F30" s="7"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="8"/>
-      <c r="J30" s="5"/>
+      <c r="H30" s="8"/>
+      <c r="I30" s="5"/>
+      <c r="J30" s="6"/>
       <c r="K30" s="6"/>
-      <c r="L30" s="6"/>
+      <c r="L30" s="8"/>
       <c r="M30" s="8"/>
-      <c r="N30" s="8"/>
-      <c r="O30" s="10"/>
-    </row>
-    <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N30" s="10"/>
+    </row>
+    <row r="31" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <v>30</v>
       </c>
@@ -2199,16 +2163,15 @@
       <c r="E31" s="5"/>
       <c r="F31" s="7"/>
       <c r="G31" s="8"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="8"/>
-      <c r="J31" s="5"/>
+      <c r="H31" s="8"/>
+      <c r="I31" s="5"/>
+      <c r="J31" s="6"/>
       <c r="K31" s="6"/>
-      <c r="L31" s="6"/>
+      <c r="L31" s="8"/>
       <c r="M31" s="8"/>
-      <c r="N31" s="8"/>
-      <c r="O31" s="10"/>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N31" s="10"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <v>31</v>
       </c>
@@ -2218,16 +2181,15 @@
       <c r="E32" s="5"/>
       <c r="F32" s="7"/>
       <c r="G32" s="8"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="8"/>
-      <c r="J32" s="5"/>
+      <c r="H32" s="8"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="6"/>
       <c r="K32" s="6"/>
-      <c r="L32" s="6"/>
+      <c r="L32" s="8"/>
       <c r="M32" s="8"/>
-      <c r="N32" s="8"/>
-      <c r="O32" s="10"/>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N32" s="10"/>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
         <v>32</v>
       </c>
@@ -2237,16 +2199,15 @@
       <c r="E33" s="5"/>
       <c r="F33" s="7"/>
       <c r="G33" s="8"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="8"/>
-      <c r="J33" s="5"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="6"/>
       <c r="K33" s="6"/>
-      <c r="L33" s="6"/>
+      <c r="L33" s="8"/>
       <c r="M33" s="8"/>
-      <c r="N33" s="8"/>
-      <c r="O33" s="10"/>
-    </row>
-    <row r="34" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N33" s="10"/>
+    </row>
+    <row r="34" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
         <v>33</v>
       </c>
@@ -2256,16 +2217,15 @@
       <c r="E34" s="5"/>
       <c r="F34" s="7"/>
       <c r="G34" s="8"/>
-      <c r="H34" s="5"/>
-      <c r="I34" s="8"/>
-      <c r="J34" s="5"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="6"/>
       <c r="K34" s="6"/>
-      <c r="L34" s="6"/>
+      <c r="L34" s="8"/>
       <c r="M34" s="8"/>
-      <c r="N34" s="8"/>
-      <c r="O34" s="10"/>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N34" s="10"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="4">
         <v>34</v>
       </c>
@@ -2275,16 +2235,15 @@
       <c r="E35" s="5"/>
       <c r="F35" s="7"/>
       <c r="G35" s="8"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="5"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="6"/>
       <c r="K35" s="6"/>
-      <c r="L35" s="6"/>
+      <c r="L35" s="8"/>
       <c r="M35" s="8"/>
-      <c r="N35" s="8"/>
-      <c r="O35" s="10"/>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N35" s="10"/>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
         <v>35</v>
       </c>
@@ -2294,16 +2253,15 @@
       <c r="E36" s="5"/>
       <c r="F36" s="7"/>
       <c r="G36" s="8"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="8"/>
-      <c r="J36" s="5"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="4"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="5"/>
+      <c r="J36" s="6"/>
+      <c r="K36" s="4"/>
+      <c r="L36" s="8"/>
       <c r="M36" s="8"/>
-      <c r="N36" s="8"/>
-      <c r="O36" s="10"/>
-    </row>
-    <row r="37" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N36" s="10"/>
+    </row>
+    <row r="37" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4">
         <v>36</v>
       </c>
@@ -2313,16 +2271,15 @@
       <c r="E37" s="5"/>
       <c r="F37" s="7"/>
       <c r="G37" s="8"/>
-      <c r="H37" s="5"/>
-      <c r="I37" s="8"/>
-      <c r="J37" s="5"/>
-      <c r="K37" s="6"/>
-      <c r="L37" s="4"/>
+      <c r="H37" s="8"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="6"/>
+      <c r="K37" s="4"/>
+      <c r="L37" s="8"/>
       <c r="M37" s="8"/>
-      <c r="N37" s="8"/>
-      <c r="O37" s="10"/>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N37" s="10"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="4">
         <v>37</v>
       </c>
@@ -2332,16 +2289,15 @@
       <c r="E38" s="5"/>
       <c r="F38" s="7"/>
       <c r="G38" s="8"/>
-      <c r="H38" s="5"/>
-      <c r="I38" s="8"/>
-      <c r="J38" s="5"/>
-      <c r="K38" s="6"/>
-      <c r="L38" s="4"/>
+      <c r="H38" s="8"/>
+      <c r="I38" s="5"/>
+      <c r="J38" s="6"/>
+      <c r="K38" s="4"/>
+      <c r="L38" s="8"/>
       <c r="M38" s="8"/>
-      <c r="N38" s="8"/>
-      <c r="O38" s="10"/>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N38" s="10"/>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="4">
         <v>38</v>
       </c>
@@ -2351,16 +2307,15 @@
       <c r="E39" s="5"/>
       <c r="F39" s="7"/>
       <c r="G39" s="8"/>
-      <c r="H39" s="5"/>
-      <c r="I39" s="8"/>
-      <c r="J39" s="5"/>
-      <c r="K39" s="6"/>
-      <c r="L39" s="4"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="5"/>
+      <c r="J39" s="6"/>
+      <c r="K39" s="4"/>
+      <c r="L39" s="8"/>
       <c r="M39" s="8"/>
-      <c r="N39" s="8"/>
-      <c r="O39" s="10"/>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N39" s="10"/>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="4">
         <v>39</v>
       </c>
@@ -2370,16 +2325,15 @@
       <c r="E40" s="5"/>
       <c r="F40" s="7"/>
       <c r="G40" s="8"/>
-      <c r="H40" s="5"/>
-      <c r="I40" s="8"/>
-      <c r="J40" s="5"/>
-      <c r="K40" s="6"/>
-      <c r="L40" s="4"/>
+      <c r="H40" s="8"/>
+      <c r="I40" s="5"/>
+      <c r="J40" s="6"/>
+      <c r="K40" s="4"/>
+      <c r="L40" s="8"/>
       <c r="M40" s="8"/>
-      <c r="N40" s="8"/>
-      <c r="O40" s="10"/>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N40" s="10"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="4">
         <v>40</v>
       </c>
@@ -2389,16 +2343,15 @@
       <c r="E41" s="5"/>
       <c r="F41" s="7"/>
       <c r="G41" s="8"/>
-      <c r="H41" s="5"/>
-      <c r="I41" s="8"/>
-      <c r="J41" s="5"/>
-      <c r="K41" s="6"/>
-      <c r="L41" s="4"/>
+      <c r="H41" s="8"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="6"/>
+      <c r="K41" s="4"/>
+      <c r="L41" s="8"/>
       <c r="M41" s="8"/>
-      <c r="N41" s="8"/>
-      <c r="O41" s="10"/>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N41" s="10"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="4">
         <v>41</v>
       </c>
@@ -2408,16 +2361,15 @@
       <c r="E42" s="5"/>
       <c r="F42" s="7"/>
       <c r="G42" s="8"/>
-      <c r="H42" s="5"/>
-      <c r="I42" s="8"/>
-      <c r="J42" s="5"/>
-      <c r="K42" s="6"/>
-      <c r="L42" s="4"/>
+      <c r="H42" s="8"/>
+      <c r="I42" s="5"/>
+      <c r="J42" s="6"/>
+      <c r="K42" s="4"/>
+      <c r="L42" s="8"/>
       <c r="M42" s="8"/>
-      <c r="N42" s="8"/>
-      <c r="O42" s="10"/>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N42" s="10"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="4">
         <v>42</v>
       </c>
@@ -2427,16 +2379,15 @@
       <c r="E43" s="5"/>
       <c r="F43" s="7"/>
       <c r="G43" s="8"/>
-      <c r="H43" s="5"/>
-      <c r="I43" s="8"/>
-      <c r="J43" s="5"/>
-      <c r="K43" s="6"/>
-      <c r="L43" s="4"/>
+      <c r="H43" s="8"/>
+      <c r="I43" s="5"/>
+      <c r="J43" s="6"/>
+      <c r="K43" s="4"/>
+      <c r="L43" s="8"/>
       <c r="M43" s="8"/>
-      <c r="N43" s="8"/>
-      <c r="O43" s="10"/>
-    </row>
-    <row r="44" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N43" s="10"/>
+    </row>
+    <row r="44" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="4">
         <v>43</v>
       </c>
@@ -2446,16 +2397,15 @@
       <c r="E44" s="5"/>
       <c r="F44" s="7"/>
       <c r="G44" s="8"/>
-      <c r="H44" s="5"/>
-      <c r="I44" s="8"/>
-      <c r="J44" s="5"/>
-      <c r="K44" s="6"/>
-      <c r="L44" s="4"/>
+      <c r="H44" s="8"/>
+      <c r="I44" s="5"/>
+      <c r="J44" s="6"/>
+      <c r="K44" s="4"/>
+      <c r="L44" s="8"/>
       <c r="M44" s="8"/>
-      <c r="N44" s="8"/>
-      <c r="O44" s="10"/>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N44" s="10"/>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="4">
         <v>44</v>
       </c>
@@ -2465,16 +2415,15 @@
       <c r="E45" s="5"/>
       <c r="F45" s="7"/>
       <c r="G45" s="8"/>
-      <c r="H45" s="5"/>
-      <c r="I45" s="8"/>
-      <c r="J45" s="5"/>
-      <c r="K45" s="6"/>
-      <c r="L45" s="4"/>
+      <c r="H45" s="8"/>
+      <c r="I45" s="5"/>
+      <c r="J45" s="6"/>
+      <c r="K45" s="4"/>
+      <c r="L45" s="8"/>
       <c r="M45" s="8"/>
-      <c r="N45" s="8"/>
-      <c r="O45" s="10"/>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N45" s="10"/>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="4">
         <v>45</v>
       </c>
@@ -2484,16 +2433,15 @@
       <c r="E46" s="5"/>
       <c r="F46" s="7"/>
       <c r="G46" s="8"/>
-      <c r="H46" s="5"/>
-      <c r="I46" s="8"/>
-      <c r="J46" s="5"/>
+      <c r="H46" s="8"/>
+      <c r="I46" s="5"/>
+      <c r="J46" s="6"/>
       <c r="K46" s="6"/>
-      <c r="L46" s="6"/>
+      <c r="L46" s="8"/>
       <c r="M46" s="8"/>
-      <c r="N46" s="8"/>
-      <c r="O46" s="10"/>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N46" s="10"/>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="4">
         <v>46</v>
       </c>
@@ -2503,16 +2451,15 @@
       <c r="E47" s="5"/>
       <c r="F47" s="7"/>
       <c r="G47" s="8"/>
-      <c r="H47" s="5"/>
-      <c r="I47" s="8"/>
-      <c r="J47" s="5"/>
+      <c r="H47" s="8"/>
+      <c r="I47" s="5"/>
+      <c r="J47" s="6"/>
       <c r="K47" s="6"/>
-      <c r="L47" s="6"/>
+      <c r="L47" s="8"/>
       <c r="M47" s="8"/>
-      <c r="N47" s="8"/>
-      <c r="O47" s="10"/>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N47" s="10"/>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="4">
         <v>47</v>
       </c>
@@ -2522,16 +2469,15 @@
       <c r="E48" s="5"/>
       <c r="F48" s="7"/>
       <c r="G48" s="8"/>
-      <c r="H48" s="5"/>
-      <c r="I48" s="8"/>
-      <c r="J48" s="5"/>
+      <c r="H48" s="8"/>
+      <c r="I48" s="5"/>
+      <c r="J48" s="6"/>
       <c r="K48" s="6"/>
-      <c r="L48" s="6"/>
+      <c r="L48" s="8"/>
       <c r="M48" s="8"/>
-      <c r="N48" s="8"/>
-      <c r="O48" s="10"/>
-    </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N48" s="10"/>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="4">
         <v>48</v>
       </c>
@@ -2541,16 +2487,15 @@
       <c r="E49" s="5"/>
       <c r="F49" s="7"/>
       <c r="G49" s="4"/>
-      <c r="H49" s="5"/>
-      <c r="I49" s="4"/>
-      <c r="J49" s="5"/>
-      <c r="K49" s="6"/>
-      <c r="L49" s="12"/>
-      <c r="M49" s="13"/>
-      <c r="N49" s="14"/>
-      <c r="O49" s="10"/>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H49" s="4"/>
+      <c r="I49" s="5"/>
+      <c r="J49" s="6"/>
+      <c r="K49" s="12"/>
+      <c r="L49" s="13"/>
+      <c r="M49" s="14"/>
+      <c r="N49" s="10"/>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" s="4">
         <v>49</v>
       </c>
@@ -2560,16 +2505,15 @@
       <c r="E50" s="5"/>
       <c r="F50" s="7"/>
       <c r="G50" s="4"/>
-      <c r="H50" s="5"/>
-      <c r="I50" s="4"/>
-      <c r="J50" s="5"/>
-      <c r="K50" s="6"/>
-      <c r="L50" s="12"/>
-      <c r="M50" s="13"/>
-      <c r="N50" s="14"/>
-      <c r="O50" s="10"/>
-    </row>
-    <row r="51" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H50" s="4"/>
+      <c r="I50" s="5"/>
+      <c r="J50" s="6"/>
+      <c r="K50" s="12"/>
+      <c r="L50" s="13"/>
+      <c r="M50" s="14"/>
+      <c r="N50" s="10"/>
+    </row>
+    <row r="51" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="4">
         <v>50</v>
       </c>
@@ -2581,14 +2525,13 @@
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
       <c r="I51" s="4"/>
-      <c r="J51" s="4"/>
-      <c r="K51" s="6"/>
-      <c r="L51" s="12"/>
-      <c r="M51" s="13"/>
-      <c r="N51" s="14"/>
-      <c r="O51" s="10"/>
-    </row>
-    <row r="52" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J51" s="6"/>
+      <c r="K51" s="12"/>
+      <c r="L51" s="13"/>
+      <c r="M51" s="14"/>
+      <c r="N51" s="10"/>
+    </row>
+    <row r="52" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="4">
         <v>51</v>
       </c>
@@ -2600,14 +2543,13 @@
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
       <c r="I52" s="4"/>
-      <c r="J52" s="4"/>
-      <c r="K52" s="6"/>
-      <c r="L52" s="12"/>
-      <c r="M52" s="13"/>
-      <c r="N52" s="14"/>
-      <c r="O52" s="10"/>
-    </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J52" s="6"/>
+      <c r="K52" s="12"/>
+      <c r="L52" s="13"/>
+      <c r="M52" s="14"/>
+      <c r="N52" s="10"/>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="4">
         <v>52</v>
       </c>
@@ -2619,14 +2561,13 @@
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
       <c r="I53" s="4"/>
-      <c r="J53" s="4"/>
-      <c r="K53" s="6"/>
-      <c r="L53" s="12"/>
-      <c r="M53" s="13"/>
-      <c r="N53" s="14"/>
-      <c r="O53" s="10"/>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J53" s="6"/>
+      <c r="K53" s="12"/>
+      <c r="L53" s="13"/>
+      <c r="M53" s="14"/>
+      <c r="N53" s="10"/>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="4">
         <v>53</v>
       </c>
@@ -2638,14 +2579,13 @@
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
       <c r="I54" s="4"/>
-      <c r="J54" s="4"/>
-      <c r="K54" s="6"/>
-      <c r="L54" s="12"/>
-      <c r="M54" s="13"/>
-      <c r="N54" s="14"/>
-      <c r="O54" s="10"/>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J54" s="6"/>
+      <c r="K54" s="12"/>
+      <c r="L54" s="13"/>
+      <c r="M54" s="14"/>
+      <c r="N54" s="10"/>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="4">
         <v>54</v>
       </c>
@@ -2657,14 +2597,13 @@
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
       <c r="I55" s="4"/>
-      <c r="J55" s="4"/>
-      <c r="K55" s="6"/>
-      <c r="L55" s="12"/>
-      <c r="M55" s="13"/>
-      <c r="N55" s="14"/>
-      <c r="O55" s="10"/>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J55" s="6"/>
+      <c r="K55" s="12"/>
+      <c r="L55" s="13"/>
+      <c r="M55" s="14"/>
+      <c r="N55" s="10"/>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="4">
         <v>55</v>
       </c>
@@ -2676,14 +2615,13 @@
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
       <c r="I56" s="4"/>
-      <c r="J56" s="4"/>
-      <c r="K56" s="6"/>
-      <c r="L56" s="12"/>
-      <c r="M56" s="13"/>
-      <c r="N56" s="14"/>
-      <c r="O56" s="10"/>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J56" s="6"/>
+      <c r="K56" s="12"/>
+      <c r="L56" s="13"/>
+      <c r="M56" s="14"/>
+      <c r="N56" s="10"/>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="4">
         <v>56</v>
       </c>
@@ -2695,14 +2633,13 @@
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
       <c r="I57" s="4"/>
-      <c r="J57" s="4"/>
-      <c r="K57" s="6"/>
-      <c r="L57" s="12"/>
-      <c r="M57" s="13"/>
-      <c r="N57" s="14"/>
-      <c r="O57" s="10"/>
-    </row>
-    <row r="58" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J57" s="6"/>
+      <c r="K57" s="12"/>
+      <c r="L57" s="13"/>
+      <c r="M57" s="14"/>
+      <c r="N57" s="10"/>
+    </row>
+    <row r="58" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="4">
         <v>57</v>
       </c>
@@ -2714,14 +2651,13 @@
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
       <c r="I58" s="4"/>
-      <c r="J58" s="4"/>
-      <c r="K58" s="6"/>
-      <c r="L58" s="12"/>
-      <c r="M58" s="13"/>
-      <c r="N58" s="14"/>
-      <c r="O58" s="10"/>
-    </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J58" s="6"/>
+      <c r="K58" s="12"/>
+      <c r="L58" s="13"/>
+      <c r="M58" s="14"/>
+      <c r="N58" s="10"/>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="4">
         <v>58</v>
       </c>
@@ -2733,14 +2669,13 @@
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
       <c r="I59" s="4"/>
-      <c r="J59" s="4"/>
-      <c r="K59" s="6"/>
-      <c r="L59" s="12"/>
-      <c r="M59" s="13"/>
-      <c r="N59" s="14"/>
-      <c r="O59" s="10"/>
-    </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J59" s="6"/>
+      <c r="K59" s="12"/>
+      <c r="L59" s="13"/>
+      <c r="M59" s="14"/>
+      <c r="N59" s="10"/>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="4">
         <v>59</v>
       </c>
@@ -2752,14 +2687,13 @@
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
       <c r="I60" s="4"/>
-      <c r="J60" s="4"/>
-      <c r="K60" s="6"/>
-      <c r="L60" s="12"/>
-      <c r="M60" s="13"/>
-      <c r="N60" s="14"/>
-      <c r="O60" s="10"/>
-    </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J60" s="6"/>
+      <c r="K60" s="12"/>
+      <c r="L60" s="13"/>
+      <c r="M60" s="14"/>
+      <c r="N60" s="10"/>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="4">
         <v>60</v>
       </c>
@@ -2771,14 +2705,13 @@
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
       <c r="I61" s="4"/>
-      <c r="J61" s="4"/>
-      <c r="K61" s="6"/>
-      <c r="L61" s="12"/>
-      <c r="M61" s="13"/>
-      <c r="N61" s="14"/>
-      <c r="O61" s="10"/>
-    </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J61" s="6"/>
+      <c r="K61" s="12"/>
+      <c r="L61" s="13"/>
+      <c r="M61" s="14"/>
+      <c r="N61" s="10"/>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="4">
         <v>61</v>
       </c>
@@ -2790,14 +2723,13 @@
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
       <c r="I62" s="4"/>
-      <c r="J62" s="4"/>
-      <c r="K62" s="6"/>
-      <c r="L62" s="12"/>
-      <c r="M62" s="13"/>
-      <c r="N62" s="14"/>
-      <c r="O62" s="10"/>
-    </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J62" s="6"/>
+      <c r="K62" s="12"/>
+      <c r="L62" s="13"/>
+      <c r="M62" s="14"/>
+      <c r="N62" s="10"/>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="4">
         <v>62</v>
       </c>
@@ -2809,14 +2741,13 @@
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
       <c r="I63" s="4"/>
-      <c r="J63" s="4"/>
-      <c r="K63" s="6"/>
-      <c r="L63" s="12"/>
-      <c r="M63" s="13"/>
-      <c r="N63" s="14"/>
-      <c r="O63" s="10"/>
-    </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J63" s="6"/>
+      <c r="K63" s="12"/>
+      <c r="L63" s="13"/>
+      <c r="M63" s="14"/>
+      <c r="N63" s="10"/>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="4">
         <v>63</v>
       </c>
@@ -2828,14 +2759,13 @@
       <c r="G64" s="4"/>
       <c r="H64" s="4"/>
       <c r="I64" s="4"/>
-      <c r="J64" s="4"/>
-      <c r="K64" s="6"/>
-      <c r="L64" s="12"/>
-      <c r="M64" s="13"/>
-      <c r="N64" s="14"/>
-      <c r="O64" s="10"/>
-    </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J64" s="6"/>
+      <c r="K64" s="12"/>
+      <c r="L64" s="13"/>
+      <c r="M64" s="14"/>
+      <c r="N64" s="10"/>
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="4">
         <v>64</v>
       </c>
@@ -2847,14 +2777,13 @@
       <c r="G65" s="4"/>
       <c r="H65" s="4"/>
       <c r="I65" s="4"/>
-      <c r="J65" s="4"/>
-      <c r="K65" s="6"/>
-      <c r="L65" s="12"/>
-      <c r="M65" s="13"/>
-      <c r="N65" s="14"/>
-      <c r="O65" s="10"/>
-    </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J65" s="6"/>
+      <c r="K65" s="12"/>
+      <c r="L65" s="13"/>
+      <c r="M65" s="14"/>
+      <c r="N65" s="10"/>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="4">
         <v>65</v>
       </c>
@@ -2866,14 +2795,13 @@
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
       <c r="I66" s="4"/>
-      <c r="J66" s="4"/>
-      <c r="K66" s="6"/>
-      <c r="L66" s="12"/>
-      <c r="M66" s="13"/>
-      <c r="N66" s="14"/>
-      <c r="O66" s="10"/>
-    </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J66" s="6"/>
+      <c r="K66" s="12"/>
+      <c r="L66" s="13"/>
+      <c r="M66" s="14"/>
+      <c r="N66" s="10"/>
+    </row>
+    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="4">
         <v>66</v>
       </c>
@@ -2885,14 +2813,13 @@
       <c r="G67" s="4"/>
       <c r="H67" s="4"/>
       <c r="I67" s="4"/>
-      <c r="J67" s="4"/>
-      <c r="K67" s="6"/>
-      <c r="L67" s="12"/>
-      <c r="M67" s="13"/>
-      <c r="N67" s="14"/>
-      <c r="O67" s="10"/>
-    </row>
-    <row r="68" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J67" s="6"/>
+      <c r="K67" s="12"/>
+      <c r="L67" s="13"/>
+      <c r="M67" s="14"/>
+      <c r="N67" s="10"/>
+    </row>
+    <row r="68" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
         <v>67</v>
       </c>
@@ -2904,14 +2831,13 @@
       <c r="G68" s="4"/>
       <c r="H68" s="4"/>
       <c r="I68" s="4"/>
-      <c r="J68" s="4"/>
-      <c r="K68" s="6"/>
-      <c r="L68" s="12"/>
-      <c r="M68" s="13"/>
-      <c r="N68" s="14"/>
-      <c r="O68" s="10"/>
-    </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J68" s="6"/>
+      <c r="K68" s="12"/>
+      <c r="L68" s="13"/>
+      <c r="M68" s="14"/>
+      <c r="N68" s="10"/>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="4">
         <v>68</v>
       </c>
@@ -2923,14 +2849,13 @@
       <c r="G69" s="4"/>
       <c r="H69" s="4"/>
       <c r="I69" s="4"/>
-      <c r="J69" s="4"/>
-      <c r="K69" s="6"/>
-      <c r="L69" s="12"/>
-      <c r="M69" s="13"/>
-      <c r="N69" s="14"/>
-      <c r="O69" s="10"/>
-    </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J69" s="6"/>
+      <c r="K69" s="12"/>
+      <c r="L69" s="13"/>
+      <c r="M69" s="14"/>
+      <c r="N69" s="10"/>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
         <v>69</v>
       </c>
@@ -2942,14 +2867,13 @@
       <c r="G70" s="4"/>
       <c r="H70" s="4"/>
       <c r="I70" s="4"/>
-      <c r="J70" s="4"/>
-      <c r="K70" s="6"/>
-      <c r="L70" s="12"/>
-      <c r="M70" s="13"/>
-      <c r="N70" s="14"/>
-      <c r="O70" s="10"/>
-    </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J70" s="6"/>
+      <c r="K70" s="12"/>
+      <c r="L70" s="13"/>
+      <c r="M70" s="14"/>
+      <c r="N70" s="10"/>
+    </row>
+    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="4">
         <v>70</v>
       </c>
@@ -2961,14 +2885,13 @@
       <c r="G71" s="4"/>
       <c r="H71" s="4"/>
       <c r="I71" s="4"/>
-      <c r="J71" s="4"/>
-      <c r="K71" s="6"/>
-      <c r="L71" s="12"/>
-      <c r="M71" s="13"/>
-      <c r="N71" s="14"/>
-      <c r="O71" s="10"/>
-    </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J71" s="6"/>
+      <c r="K71" s="12"/>
+      <c r="L71" s="13"/>
+      <c r="M71" s="14"/>
+      <c r="N71" s="10"/>
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" s="4">
         <v>71</v>
       </c>
@@ -2980,14 +2903,13 @@
       <c r="G72" s="4"/>
       <c r="H72" s="4"/>
       <c r="I72" s="4"/>
-      <c r="J72" s="4"/>
-      <c r="K72" s="6"/>
-      <c r="L72" s="12"/>
-      <c r="M72" s="13"/>
-      <c r="N72" s="14"/>
-      <c r="O72" s="10"/>
-    </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J72" s="6"/>
+      <c r="K72" s="12"/>
+      <c r="L72" s="13"/>
+      <c r="M72" s="14"/>
+      <c r="N72" s="10"/>
+    </row>
+    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" s="4">
         <v>72</v>
       </c>
@@ -2999,14 +2921,13 @@
       <c r="G73" s="4"/>
       <c r="H73" s="4"/>
       <c r="I73" s="4"/>
-      <c r="J73" s="4"/>
-      <c r="K73" s="6"/>
-      <c r="L73" s="12"/>
-      <c r="M73" s="13"/>
-      <c r="N73" s="14"/>
-      <c r="O73" s="10"/>
-    </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J73" s="6"/>
+      <c r="K73" s="12"/>
+      <c r="L73" s="13"/>
+      <c r="M73" s="14"/>
+      <c r="N73" s="10"/>
+    </row>
+    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A74" s="4">
         <v>73</v>
       </c>
@@ -3018,14 +2939,13 @@
       <c r="G74" s="4"/>
       <c r="H74" s="4"/>
       <c r="I74" s="4"/>
-      <c r="J74" s="4"/>
-      <c r="K74" s="6"/>
-      <c r="L74" s="12"/>
-      <c r="M74" s="13"/>
-      <c r="N74" s="14"/>
-      <c r="O74" s="10"/>
-    </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J74" s="6"/>
+      <c r="K74" s="12"/>
+      <c r="L74" s="13"/>
+      <c r="M74" s="14"/>
+      <c r="N74" s="10"/>
+    </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A75" s="4">
         <v>74</v>
       </c>
@@ -3037,14 +2957,13 @@
       <c r="G75" s="4"/>
       <c r="H75" s="4"/>
       <c r="I75" s="4"/>
-      <c r="J75" s="4"/>
-      <c r="K75" s="6"/>
-      <c r="L75" s="12"/>
-      <c r="M75" s="13"/>
-      <c r="N75" s="14"/>
-      <c r="O75" s="10"/>
-    </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J75" s="6"/>
+      <c r="K75" s="12"/>
+      <c r="L75" s="13"/>
+      <c r="M75" s="14"/>
+      <c r="N75" s="10"/>
+    </row>
+    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A76" s="4">
         <v>75</v>
       </c>
@@ -3056,14 +2975,13 @@
       <c r="G76" s="4"/>
       <c r="H76" s="4"/>
       <c r="I76" s="4"/>
-      <c r="J76" s="4"/>
-      <c r="K76" s="6"/>
-      <c r="L76" s="12"/>
-      <c r="M76" s="13"/>
-      <c r="N76" s="14"/>
-      <c r="O76" s="10"/>
-    </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J76" s="6"/>
+      <c r="K76" s="12"/>
+      <c r="L76" s="13"/>
+      <c r="M76" s="14"/>
+      <c r="N76" s="10"/>
+    </row>
+    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A77" s="4">
         <v>76</v>
       </c>
@@ -3075,14 +2993,13 @@
       <c r="G77" s="4"/>
       <c r="H77" s="4"/>
       <c r="I77" s="4"/>
-      <c r="J77" s="4"/>
-      <c r="K77" s="6"/>
-      <c r="L77" s="12"/>
-      <c r="M77" s="13"/>
-      <c r="N77" s="14"/>
-      <c r="O77" s="10"/>
-    </row>
-    <row r="78" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J77" s="6"/>
+      <c r="K77" s="12"/>
+      <c r="L77" s="13"/>
+      <c r="M77" s="14"/>
+      <c r="N77" s="10"/>
+    </row>
+    <row r="78" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="4">
         <v>77</v>
       </c>
@@ -3094,14 +3011,13 @@
       <c r="G78" s="4"/>
       <c r="H78" s="4"/>
       <c r="I78" s="4"/>
-      <c r="J78" s="4"/>
-      <c r="K78" s="6"/>
-      <c r="L78" s="12"/>
-      <c r="M78" s="13"/>
-      <c r="N78" s="14"/>
-      <c r="O78" s="10"/>
-    </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J78" s="6"/>
+      <c r="K78" s="12"/>
+      <c r="L78" s="13"/>
+      <c r="M78" s="14"/>
+      <c r="N78" s="10"/>
+    </row>
+    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A79" s="4">
         <v>78</v>
       </c>
@@ -3113,14 +3029,13 @@
       <c r="G79" s="4"/>
       <c r="H79" s="4"/>
       <c r="I79" s="4"/>
-      <c r="J79" s="4"/>
-      <c r="K79" s="6"/>
-      <c r="L79" s="12"/>
-      <c r="M79" s="13"/>
-      <c r="N79" s="14"/>
-      <c r="O79" s="10"/>
-    </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J79" s="6"/>
+      <c r="K79" s="12"/>
+      <c r="L79" s="13"/>
+      <c r="M79" s="14"/>
+      <c r="N79" s="10"/>
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
         <v>79</v>
       </c>
@@ -3132,14 +3047,13 @@
       <c r="G80" s="4"/>
       <c r="H80" s="4"/>
       <c r="I80" s="4"/>
-      <c r="J80" s="4"/>
-      <c r="K80" s="6"/>
-      <c r="L80" s="12"/>
-      <c r="M80" s="13"/>
-      <c r="N80" s="14"/>
-      <c r="O80" s="10"/>
-    </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J80" s="6"/>
+      <c r="K80" s="12"/>
+      <c r="L80" s="13"/>
+      <c r="M80" s="14"/>
+      <c r="N80" s="10"/>
+    </row>
+    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A81" s="4">
         <v>80</v>
       </c>
@@ -3151,14 +3065,13 @@
       <c r="G81" s="4"/>
       <c r="H81" s="4"/>
       <c r="I81" s="4"/>
-      <c r="J81" s="4"/>
-      <c r="K81" s="6"/>
-      <c r="L81" s="12"/>
-      <c r="M81" s="13"/>
-      <c r="N81" s="14"/>
-      <c r="O81" s="10"/>
-    </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J81" s="6"/>
+      <c r="K81" s="12"/>
+      <c r="L81" s="13"/>
+      <c r="M81" s="14"/>
+      <c r="N81" s="10"/>
+    </row>
+    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
         <v>81</v>
       </c>
@@ -3170,14 +3083,13 @@
       <c r="G82" s="4"/>
       <c r="H82" s="4"/>
       <c r="I82" s="4"/>
-      <c r="J82" s="4"/>
-      <c r="K82" s="6"/>
-      <c r="L82" s="12"/>
-      <c r="M82" s="13"/>
-      <c r="N82" s="14"/>
-      <c r="O82" s="10"/>
-    </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J82" s="6"/>
+      <c r="K82" s="12"/>
+      <c r="L82" s="13"/>
+      <c r="M82" s="14"/>
+      <c r="N82" s="10"/>
+    </row>
+    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A83" s="4">
         <v>82</v>
       </c>
@@ -3189,14 +3101,13 @@
       <c r="G83" s="4"/>
       <c r="H83" s="4"/>
       <c r="I83" s="4"/>
-      <c r="J83" s="4"/>
-      <c r="K83" s="6"/>
-      <c r="L83" s="12"/>
-      <c r="M83" s="13"/>
-      <c r="N83" s="14"/>
-      <c r="O83" s="10"/>
-    </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J83" s="6"/>
+      <c r="K83" s="12"/>
+      <c r="L83" s="13"/>
+      <c r="M83" s="14"/>
+      <c r="N83" s="10"/>
+    </row>
+    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
         <v>83</v>
       </c>
@@ -3208,14 +3119,13 @@
       <c r="G84" s="4"/>
       <c r="H84" s="4"/>
       <c r="I84" s="4"/>
-      <c r="J84" s="4"/>
-      <c r="K84" s="6"/>
-      <c r="L84" s="12"/>
-      <c r="M84" s="13"/>
-      <c r="N84" s="14"/>
-      <c r="O84" s="10"/>
-    </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J84" s="6"/>
+      <c r="K84" s="12"/>
+      <c r="L84" s="13"/>
+      <c r="M84" s="14"/>
+      <c r="N84" s="10"/>
+    </row>
+    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A85" s="4">
         <v>84</v>
       </c>
@@ -3227,14 +3137,13 @@
       <c r="G85" s="4"/>
       <c r="H85" s="4"/>
       <c r="I85" s="4"/>
-      <c r="J85" s="4"/>
-      <c r="K85" s="6"/>
-      <c r="L85" s="12"/>
-      <c r="M85" s="13"/>
-      <c r="N85" s="14"/>
-      <c r="O85" s="10"/>
-    </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J85" s="6"/>
+      <c r="K85" s="12"/>
+      <c r="L85" s="13"/>
+      <c r="M85" s="14"/>
+      <c r="N85" s="10"/>
+    </row>
+    <row r="86" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A86" s="4">
         <v>85</v>
       </c>
@@ -3246,14 +3155,13 @@
       <c r="G86" s="4"/>
       <c r="H86" s="4"/>
       <c r="I86" s="4"/>
-      <c r="J86" s="4"/>
-      <c r="K86" s="6"/>
-      <c r="L86" s="12"/>
-      <c r="M86" s="13"/>
-      <c r="N86" s="14"/>
-      <c r="O86" s="10"/>
-    </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J86" s="6"/>
+      <c r="K86" s="12"/>
+      <c r="L86" s="13"/>
+      <c r="M86" s="14"/>
+      <c r="N86" s="10"/>
+    </row>
+    <row r="87" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A87" s="4">
         <v>86</v>
       </c>
@@ -3265,14 +3173,13 @@
       <c r="G87" s="4"/>
       <c r="H87" s="4"/>
       <c r="I87" s="4"/>
-      <c r="J87" s="4"/>
-      <c r="K87" s="6"/>
-      <c r="L87" s="12"/>
-      <c r="M87" s="13"/>
-      <c r="N87" s="14"/>
-      <c r="O87" s="10"/>
-    </row>
-    <row r="88" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J87" s="6"/>
+      <c r="K87" s="12"/>
+      <c r="L87" s="13"/>
+      <c r="M87" s="14"/>
+      <c r="N87" s="10"/>
+    </row>
+    <row r="88" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="4">
         <v>87</v>
       </c>
@@ -3284,14 +3191,13 @@
       <c r="G88" s="4"/>
       <c r="H88" s="4"/>
       <c r="I88" s="4"/>
-      <c r="J88" s="4"/>
-      <c r="K88" s="6"/>
-      <c r="L88" s="12"/>
-      <c r="M88" s="13"/>
-      <c r="N88" s="14"/>
-      <c r="O88" s="10"/>
-    </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J88" s="6"/>
+      <c r="K88" s="12"/>
+      <c r="L88" s="13"/>
+      <c r="M88" s="14"/>
+      <c r="N88" s="10"/>
+    </row>
+    <row r="89" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A89" s="4">
         <v>88</v>
       </c>
@@ -3303,14 +3209,13 @@
       <c r="G89" s="4"/>
       <c r="H89" s="4"/>
       <c r="I89" s="4"/>
-      <c r="J89" s="4"/>
-      <c r="K89" s="6"/>
-      <c r="L89" s="12"/>
-      <c r="M89" s="13"/>
-      <c r="N89" s="14"/>
-      <c r="O89" s="10"/>
-    </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J89" s="6"/>
+      <c r="K89" s="12"/>
+      <c r="L89" s="13"/>
+      <c r="M89" s="14"/>
+      <c r="N89" s="10"/>
+    </row>
+    <row r="90" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A90" s="4">
         <v>89</v>
       </c>
@@ -3322,14 +3227,13 @@
       <c r="G90" s="4"/>
       <c r="H90" s="4"/>
       <c r="I90" s="4"/>
-      <c r="J90" s="4"/>
-      <c r="K90" s="6"/>
-      <c r="L90" s="12"/>
-      <c r="M90" s="13"/>
-      <c r="N90" s="14"/>
-      <c r="O90" s="10"/>
-    </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J90" s="6"/>
+      <c r="K90" s="12"/>
+      <c r="L90" s="13"/>
+      <c r="M90" s="14"/>
+      <c r="N90" s="10"/>
+    </row>
+    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A91" s="4">
         <v>90</v>
       </c>
@@ -3341,14 +3245,13 @@
       <c r="G91" s="4"/>
       <c r="H91" s="4"/>
       <c r="I91" s="4"/>
-      <c r="J91" s="4"/>
-      <c r="K91" s="6"/>
-      <c r="L91" s="12"/>
-      <c r="M91" s="13"/>
-      <c r="N91" s="14"/>
-      <c r="O91" s="10"/>
-    </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J91" s="6"/>
+      <c r="K91" s="12"/>
+      <c r="L91" s="13"/>
+      <c r="M91" s="14"/>
+      <c r="N91" s="10"/>
+    </row>
+    <row r="92" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A92" s="4">
         <v>91</v>
       </c>
@@ -3360,14 +3263,13 @@
       <c r="G92" s="4"/>
       <c r="H92" s="4"/>
       <c r="I92" s="4"/>
-      <c r="J92" s="4"/>
-      <c r="K92" s="6"/>
-      <c r="L92" s="12"/>
-      <c r="M92" s="13"/>
-      <c r="N92" s="14"/>
-      <c r="O92" s="10"/>
-    </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J92" s="6"/>
+      <c r="K92" s="12"/>
+      <c r="L92" s="13"/>
+      <c r="M92" s="14"/>
+      <c r="N92" s="10"/>
+    </row>
+    <row r="93" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A93" s="4">
         <v>92</v>
       </c>
@@ -3379,14 +3281,13 @@
       <c r="G93" s="4"/>
       <c r="H93" s="4"/>
       <c r="I93" s="4"/>
-      <c r="J93" s="4"/>
-      <c r="K93" s="6"/>
-      <c r="L93" s="12"/>
-      <c r="M93" s="13"/>
-      <c r="N93" s="14"/>
-      <c r="O93" s="10"/>
-    </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J93" s="6"/>
+      <c r="K93" s="12"/>
+      <c r="L93" s="13"/>
+      <c r="M93" s="14"/>
+      <c r="N93" s="10"/>
+    </row>
+    <row r="94" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A94" s="4">
         <v>93</v>
       </c>
@@ -3398,14 +3299,13 @@
       <c r="G94" s="4"/>
       <c r="H94" s="4"/>
       <c r="I94" s="4"/>
-      <c r="J94" s="4"/>
-      <c r="K94" s="6"/>
-      <c r="L94" s="12"/>
-      <c r="M94" s="13"/>
-      <c r="N94" s="14"/>
-      <c r="O94" s="10"/>
-    </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J94" s="6"/>
+      <c r="K94" s="12"/>
+      <c r="L94" s="13"/>
+      <c r="M94" s="14"/>
+      <c r="N94" s="10"/>
+    </row>
+    <row r="95" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A95" s="4">
         <v>94</v>
       </c>
@@ -3417,14 +3317,13 @@
       <c r="G95" s="4"/>
       <c r="H95" s="4"/>
       <c r="I95" s="4"/>
-      <c r="J95" s="4"/>
-      <c r="K95" s="6"/>
-      <c r="L95" s="12"/>
-      <c r="M95" s="13"/>
-      <c r="N95" s="14"/>
-      <c r="O95" s="10"/>
-    </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J95" s="6"/>
+      <c r="K95" s="12"/>
+      <c r="L95" s="13"/>
+      <c r="M95" s="14"/>
+      <c r="N95" s="10"/>
+    </row>
+    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A96" s="4">
         <v>95</v>
       </c>
@@ -3436,14 +3335,13 @@
       <c r="G96" s="4"/>
       <c r="H96" s="4"/>
       <c r="I96" s="4"/>
-      <c r="J96" s="4"/>
-      <c r="K96" s="6"/>
-      <c r="L96" s="12"/>
-      <c r="M96" s="13"/>
-      <c r="N96" s="14"/>
-      <c r="O96" s="10"/>
-    </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J96" s="6"/>
+      <c r="K96" s="12"/>
+      <c r="L96" s="13"/>
+      <c r="M96" s="14"/>
+      <c r="N96" s="10"/>
+    </row>
+    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A97" s="4">
         <v>96</v>
       </c>
@@ -3455,14 +3353,13 @@
       <c r="G97" s="4"/>
       <c r="H97" s="4"/>
       <c r="I97" s="4"/>
-      <c r="J97" s="4"/>
-      <c r="K97" s="6"/>
-      <c r="L97" s="12"/>
-      <c r="M97" s="13"/>
-      <c r="N97" s="14"/>
-      <c r="O97" s="10"/>
-    </row>
-    <row r="98" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J97" s="6"/>
+      <c r="K97" s="12"/>
+      <c r="L97" s="13"/>
+      <c r="M97" s="14"/>
+      <c r="N97" s="10"/>
+    </row>
+    <row r="98" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="4">
         <v>97</v>
       </c>
@@ -3474,14 +3371,13 @@
       <c r="G98" s="4"/>
       <c r="H98" s="4"/>
       <c r="I98" s="4"/>
-      <c r="J98" s="4"/>
-      <c r="K98" s="6"/>
-      <c r="L98" s="12"/>
-      <c r="M98" s="13"/>
-      <c r="N98" s="14"/>
-      <c r="O98" s="10"/>
-    </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J98" s="6"/>
+      <c r="K98" s="12"/>
+      <c r="L98" s="13"/>
+      <c r="M98" s="14"/>
+      <c r="N98" s="10"/>
+    </row>
+    <row r="99" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A99" s="4">
         <v>98</v>
       </c>
@@ -3493,14 +3389,13 @@
       <c r="G99" s="4"/>
       <c r="H99" s="4"/>
       <c r="I99" s="4"/>
-      <c r="J99" s="4"/>
-      <c r="K99" s="6"/>
-      <c r="L99" s="12"/>
-      <c r="M99" s="13"/>
-      <c r="N99" s="14"/>
-      <c r="O99" s="10"/>
-    </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J99" s="6"/>
+      <c r="K99" s="12"/>
+      <c r="L99" s="13"/>
+      <c r="M99" s="14"/>
+      <c r="N99" s="10"/>
+    </row>
+    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
         <v>99</v>
       </c>
@@ -3512,14 +3407,13 @@
       <c r="G100" s="4"/>
       <c r="H100" s="4"/>
       <c r="I100" s="4"/>
-      <c r="J100" s="4"/>
-      <c r="K100" s="6"/>
-      <c r="L100" s="12"/>
-      <c r="M100" s="13"/>
-      <c r="N100" s="14"/>
-      <c r="O100" s="10"/>
-    </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J100" s="6"/>
+      <c r="K100" s="12"/>
+      <c r="L100" s="13"/>
+      <c r="M100" s="14"/>
+      <c r="N100" s="10"/>
+    </row>
+    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
         <v>100</v>
       </c>
@@ -3531,14 +3425,13 @@
       <c r="G101" s="4"/>
       <c r="H101" s="4"/>
       <c r="I101" s="4"/>
-      <c r="J101" s="4"/>
-      <c r="K101" s="6"/>
-      <c r="L101" s="12"/>
-      <c r="M101" s="13"/>
-      <c r="N101" s="14"/>
-      <c r="O101" s="10"/>
-    </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J101" s="6"/>
+      <c r="K101" s="12"/>
+      <c r="L101" s="13"/>
+      <c r="M101" s="14"/>
+      <c r="N101" s="10"/>
+    </row>
+    <row r="102" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
         <v>101</v>
       </c>
@@ -3550,14 +3443,13 @@
       <c r="G102" s="4"/>
       <c r="H102" s="4"/>
       <c r="I102" s="4"/>
-      <c r="J102" s="4"/>
-      <c r="K102" s="6"/>
-      <c r="L102" s="12"/>
-      <c r="M102" s="13"/>
-      <c r="N102" s="14"/>
-      <c r="O102" s="10"/>
-    </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J102" s="6"/>
+      <c r="K102" s="12"/>
+      <c r="L102" s="13"/>
+      <c r="M102" s="14"/>
+      <c r="N102" s="10"/>
+    </row>
+    <row r="103" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
         <v>102</v>
       </c>
@@ -3569,14 +3461,13 @@
       <c r="G103" s="4"/>
       <c r="H103" s="4"/>
       <c r="I103" s="4"/>
-      <c r="J103" s="4"/>
-      <c r="K103" s="6"/>
-      <c r="L103" s="12"/>
-      <c r="M103" s="13"/>
-      <c r="N103" s="14"/>
-      <c r="O103" s="10"/>
-    </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J103" s="6"/>
+      <c r="K103" s="12"/>
+      <c r="L103" s="13"/>
+      <c r="M103" s="14"/>
+      <c r="N103" s="10"/>
+    </row>
+    <row r="104" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
         <v>103</v>
       </c>
@@ -3588,14 +3479,13 @@
       <c r="G104" s="4"/>
       <c r="H104" s="4"/>
       <c r="I104" s="4"/>
-      <c r="J104" s="4"/>
-      <c r="K104" s="6"/>
-      <c r="L104" s="12"/>
-      <c r="M104" s="13"/>
-      <c r="N104" s="14"/>
-      <c r="O104" s="10"/>
-    </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J104" s="6"/>
+      <c r="K104" s="12"/>
+      <c r="L104" s="13"/>
+      <c r="M104" s="14"/>
+      <c r="N104" s="10"/>
+    </row>
+    <row r="105" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
         <v>104</v>
       </c>
@@ -3607,14 +3497,13 @@
       <c r="G105" s="4"/>
       <c r="H105" s="4"/>
       <c r="I105" s="4"/>
-      <c r="J105" s="4"/>
-      <c r="K105" s="6"/>
-      <c r="L105" s="12"/>
-      <c r="M105" s="13"/>
-      <c r="N105" s="14"/>
-      <c r="O105" s="10"/>
-    </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J105" s="6"/>
+      <c r="K105" s="12"/>
+      <c r="L105" s="13"/>
+      <c r="M105" s="14"/>
+      <c r="N105" s="10"/>
+    </row>
+    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A106" s="4">
         <v>105</v>
       </c>
@@ -3626,14 +3515,13 @@
       <c r="G106" s="4"/>
       <c r="H106" s="4"/>
       <c r="I106" s="4"/>
-      <c r="J106" s="4"/>
-      <c r="K106" s="6"/>
-      <c r="L106" s="12"/>
-      <c r="M106" s="13"/>
-      <c r="N106" s="14"/>
-      <c r="O106" s="10"/>
-    </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J106" s="6"/>
+      <c r="K106" s="12"/>
+      <c r="L106" s="13"/>
+      <c r="M106" s="14"/>
+      <c r="N106" s="10"/>
+    </row>
+    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
         <v>106</v>
       </c>
@@ -3645,14 +3533,13 @@
       <c r="G107" s="4"/>
       <c r="H107" s="4"/>
       <c r="I107" s="4"/>
-      <c r="J107" s="4"/>
-      <c r="K107" s="6"/>
-      <c r="L107" s="12"/>
-      <c r="M107" s="13"/>
-      <c r="N107" s="14"/>
-      <c r="O107" s="10"/>
-    </row>
-    <row r="108" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J107" s="6"/>
+      <c r="K107" s="12"/>
+      <c r="L107" s="13"/>
+      <c r="M107" s="14"/>
+      <c r="N107" s="10"/>
+    </row>
+    <row r="108" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
         <v>107</v>
       </c>
@@ -3664,14 +3551,13 @@
       <c r="G108" s="4"/>
       <c r="H108" s="4"/>
       <c r="I108" s="4"/>
-      <c r="J108" s="4"/>
-      <c r="K108" s="6"/>
-      <c r="L108" s="12"/>
-      <c r="M108" s="13"/>
-      <c r="N108" s="14"/>
-      <c r="O108" s="10"/>
-    </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J108" s="6"/>
+      <c r="K108" s="12"/>
+      <c r="L108" s="13"/>
+      <c r="M108" s="14"/>
+      <c r="N108" s="10"/>
+    </row>
+    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
         <v>108</v>
       </c>
@@ -3683,14 +3569,13 @@
       <c r="G109" s="4"/>
       <c r="H109" s="4"/>
       <c r="I109" s="4"/>
-      <c r="J109" s="4"/>
-      <c r="K109" s="6"/>
-      <c r="L109" s="12"/>
-      <c r="M109" s="13"/>
-      <c r="N109" s="14"/>
-      <c r="O109" s="10"/>
-    </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J109" s="6"/>
+      <c r="K109" s="12"/>
+      <c r="L109" s="13"/>
+      <c r="M109" s="14"/>
+      <c r="N109" s="10"/>
+    </row>
+    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
         <v>109</v>
       </c>
@@ -3702,14 +3587,13 @@
       <c r="G110" s="4"/>
       <c r="H110" s="4"/>
       <c r="I110" s="4"/>
-      <c r="J110" s="4"/>
-      <c r="K110" s="6"/>
-      <c r="L110" s="12"/>
-      <c r="M110" s="13"/>
-      <c r="N110" s="14"/>
-      <c r="O110" s="10"/>
-    </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J110" s="6"/>
+      <c r="K110" s="12"/>
+      <c r="L110" s="13"/>
+      <c r="M110" s="14"/>
+      <c r="N110" s="10"/>
+    </row>
+    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
         <v>110</v>
       </c>
@@ -3721,14 +3605,13 @@
       <c r="G111" s="4"/>
       <c r="H111" s="4"/>
       <c r="I111" s="4"/>
-      <c r="J111" s="4"/>
-      <c r="K111" s="6"/>
-      <c r="L111" s="12"/>
-      <c r="M111" s="13"/>
-      <c r="N111" s="14"/>
-      <c r="O111" s="10"/>
-    </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J111" s="6"/>
+      <c r="K111" s="12"/>
+      <c r="L111" s="13"/>
+      <c r="M111" s="14"/>
+      <c r="N111" s="10"/>
+    </row>
+    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
         <v>111</v>
       </c>
@@ -3740,14 +3623,13 @@
       <c r="G112" s="4"/>
       <c r="H112" s="4"/>
       <c r="I112" s="4"/>
-      <c r="J112" s="4"/>
-      <c r="K112" s="6"/>
-      <c r="L112" s="12"/>
-      <c r="M112" s="13"/>
-      <c r="N112" s="14"/>
-      <c r="O112" s="10"/>
-    </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J112" s="6"/>
+      <c r="K112" s="12"/>
+      <c r="L112" s="13"/>
+      <c r="M112" s="14"/>
+      <c r="N112" s="10"/>
+    </row>
+    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A113" s="4">
         <v>112</v>
       </c>
@@ -3759,14 +3641,13 @@
       <c r="G113" s="4"/>
       <c r="H113" s="4"/>
       <c r="I113" s="4"/>
-      <c r="J113" s="4"/>
-      <c r="K113" s="6"/>
-      <c r="L113" s="12"/>
-      <c r="M113" s="13"/>
-      <c r="N113" s="14"/>
-      <c r="O113" s="10"/>
-    </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J113" s="6"/>
+      <c r="K113" s="12"/>
+      <c r="L113" s="13"/>
+      <c r="M113" s="14"/>
+      <c r="N113" s="10"/>
+    </row>
+    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A114" s="4">
         <v>113</v>
       </c>
@@ -3778,14 +3659,13 @@
       <c r="G114" s="4"/>
       <c r="H114" s="4"/>
       <c r="I114" s="4"/>
-      <c r="J114" s="4"/>
-      <c r="K114" s="6"/>
-      <c r="L114" s="12"/>
-      <c r="M114" s="13"/>
-      <c r="N114" s="14"/>
-      <c r="O114" s="10"/>
-    </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J114" s="6"/>
+      <c r="K114" s="12"/>
+      <c r="L114" s="13"/>
+      <c r="M114" s="14"/>
+      <c r="N114" s="10"/>
+    </row>
+    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A115" s="4">
         <v>114</v>
       </c>
@@ -3797,14 +3677,13 @@
       <c r="G115" s="4"/>
       <c r="H115" s="4"/>
       <c r="I115" s="4"/>
-      <c r="J115" s="4"/>
-      <c r="K115" s="6"/>
-      <c r="L115" s="12"/>
-      <c r="M115" s="13"/>
-      <c r="N115" s="14"/>
-      <c r="O115" s="10"/>
-    </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J115" s="6"/>
+      <c r="K115" s="12"/>
+      <c r="L115" s="13"/>
+      <c r="M115" s="14"/>
+      <c r="N115" s="10"/>
+    </row>
+    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A116" s="4">
         <v>115</v>
       </c>
@@ -3816,14 +3695,13 @@
       <c r="G116" s="4"/>
       <c r="H116" s="4"/>
       <c r="I116" s="4"/>
-      <c r="J116" s="4"/>
-      <c r="K116" s="6"/>
-      <c r="L116" s="12"/>
-      <c r="M116" s="13"/>
-      <c r="N116" s="14"/>
-      <c r="O116" s="10"/>
-    </row>
-    <row r="117" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J116" s="6"/>
+      <c r="K116" s="12"/>
+      <c r="L116" s="13"/>
+      <c r="M116" s="14"/>
+      <c r="N116" s="10"/>
+    </row>
+    <row r="117" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="4">
         <v>116</v>
       </c>
@@ -3835,14 +3713,13 @@
       <c r="G117" s="4"/>
       <c r="H117" s="4"/>
       <c r="I117" s="4"/>
-      <c r="J117" s="4"/>
-      <c r="K117" s="6"/>
-      <c r="L117" s="12"/>
-      <c r="M117" s="13"/>
-      <c r="N117" s="14"/>
-      <c r="O117" s="10"/>
-    </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J117" s="6"/>
+      <c r="K117" s="12"/>
+      <c r="L117" s="13"/>
+      <c r="M117" s="14"/>
+      <c r="N117" s="10"/>
+    </row>
+    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A118" s="4">
         <v>117</v>
       </c>
@@ -3854,14 +3731,13 @@
       <c r="G118" s="4"/>
       <c r="H118" s="4"/>
       <c r="I118" s="4"/>
-      <c r="J118" s="4"/>
-      <c r="K118" s="6"/>
-      <c r="L118" s="12"/>
-      <c r="M118" s="13"/>
-      <c r="N118" s="14"/>
-      <c r="O118" s="10"/>
-    </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J118" s="6"/>
+      <c r="K118" s="12"/>
+      <c r="L118" s="13"/>
+      <c r="M118" s="14"/>
+      <c r="N118" s="10"/>
+    </row>
+    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A119" s="4">
         <v>118</v>
       </c>
@@ -3873,14 +3749,13 @@
       <c r="G119" s="4"/>
       <c r="H119" s="4"/>
       <c r="I119" s="4"/>
-      <c r="J119" s="4"/>
-      <c r="K119" s="6"/>
-      <c r="L119" s="12"/>
-      <c r="M119" s="13"/>
-      <c r="N119" s="14"/>
-      <c r="O119" s="10"/>
-    </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J119" s="6"/>
+      <c r="K119" s="12"/>
+      <c r="L119" s="13"/>
+      <c r="M119" s="14"/>
+      <c r="N119" s="10"/>
+    </row>
+    <row r="120" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A120" s="4">
         <v>119</v>
       </c>
@@ -3892,14 +3767,13 @@
       <c r="G120" s="4"/>
       <c r="H120" s="4"/>
       <c r="I120" s="4"/>
-      <c r="J120" s="4"/>
-      <c r="K120" s="6"/>
-      <c r="L120" s="12"/>
-      <c r="M120" s="13"/>
-      <c r="N120" s="14"/>
-      <c r="O120" s="10"/>
-    </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J120" s="6"/>
+      <c r="K120" s="12"/>
+      <c r="L120" s="13"/>
+      <c r="M120" s="14"/>
+      <c r="N120" s="10"/>
+    </row>
+    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A121" s="4">
         <v>120</v>
       </c>
@@ -3911,14 +3785,13 @@
       <c r="G121" s="4"/>
       <c r="H121" s="4"/>
       <c r="I121" s="4"/>
-      <c r="J121" s="4"/>
-      <c r="K121" s="6"/>
-      <c r="L121" s="12"/>
-      <c r="M121" s="13"/>
-      <c r="N121" s="14"/>
-      <c r="O121" s="10"/>
-    </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J121" s="6"/>
+      <c r="K121" s="12"/>
+      <c r="L121" s="13"/>
+      <c r="M121" s="14"/>
+      <c r="N121" s="10"/>
+    </row>
+    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A122" s="4">
         <v>121</v>
       </c>
@@ -3930,14 +3803,13 @@
       <c r="G122" s="4"/>
       <c r="H122" s="4"/>
       <c r="I122" s="4"/>
-      <c r="J122" s="4"/>
-      <c r="K122" s="6"/>
-      <c r="L122" s="12"/>
-      <c r="M122" s="13"/>
-      <c r="N122" s="14"/>
-      <c r="O122" s="10"/>
-    </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J122" s="6"/>
+      <c r="K122" s="12"/>
+      <c r="L122" s="13"/>
+      <c r="M122" s="14"/>
+      <c r="N122" s="10"/>
+    </row>
+    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A123" s="4">
         <v>122</v>
       </c>
@@ -3949,14 +3821,13 @@
       <c r="G123" s="4"/>
       <c r="H123" s="4"/>
       <c r="I123" s="4"/>
-      <c r="J123" s="4"/>
-      <c r="K123" s="6"/>
-      <c r="L123" s="12"/>
-      <c r="M123" s="13"/>
-      <c r="N123" s="14"/>
-      <c r="O123" s="10"/>
-    </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J123" s="6"/>
+      <c r="K123" s="12"/>
+      <c r="L123" s="13"/>
+      <c r="M123" s="14"/>
+      <c r="N123" s="10"/>
+    </row>
+    <row r="124" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
         <v>123</v>
       </c>
@@ -3968,14 +3839,13 @@
       <c r="G124" s="4"/>
       <c r="H124" s="4"/>
       <c r="I124" s="4"/>
-      <c r="J124" s="4"/>
-      <c r="K124" s="6"/>
-      <c r="L124" s="12"/>
-      <c r="M124" s="13"/>
-      <c r="N124" s="14"/>
-      <c r="O124" s="10"/>
-    </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J124" s="6"/>
+      <c r="K124" s="12"/>
+      <c r="L124" s="13"/>
+      <c r="M124" s="14"/>
+      <c r="N124" s="10"/>
+    </row>
+    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
         <v>124</v>
       </c>
@@ -3987,14 +3857,13 @@
       <c r="G125" s="4"/>
       <c r="H125" s="4"/>
       <c r="I125" s="4"/>
-      <c r="J125" s="4"/>
-      <c r="K125" s="6"/>
-      <c r="L125" s="12"/>
-      <c r="M125" s="13"/>
-      <c r="N125" s="14"/>
-      <c r="O125" s="10"/>
-    </row>
-    <row r="126" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J125" s="6"/>
+      <c r="K125" s="12"/>
+      <c r="L125" s="13"/>
+      <c r="M125" s="14"/>
+      <c r="N125" s="10"/>
+    </row>
+    <row r="126" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
         <v>125</v>
       </c>
@@ -4006,14 +3875,13 @@
       <c r="G126" s="4"/>
       <c r="H126" s="4"/>
       <c r="I126" s="4"/>
-      <c r="J126" s="4"/>
-      <c r="K126" s="6"/>
-      <c r="L126" s="12"/>
-      <c r="M126" s="13"/>
-      <c r="N126" s="14"/>
-      <c r="O126" s="10"/>
-    </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J126" s="6"/>
+      <c r="K126" s="12"/>
+      <c r="L126" s="13"/>
+      <c r="M126" s="14"/>
+      <c r="N126" s="10"/>
+    </row>
+    <row r="127" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A127" s="4">
         <v>126</v>
       </c>
@@ -4025,156 +3893,155 @@
       <c r="G127" s="16"/>
       <c r="H127" s="16"/>
       <c r="I127" s="16"/>
-      <c r="J127" s="16"/>
-      <c r="K127" s="17"/>
+      <c r="J127" s="17"/>
+      <c r="K127" s="16"/>
       <c r="L127" s="16"/>
       <c r="M127" s="16"/>
-      <c r="N127" s="16"/>
-      <c r="O127" s="18"/>
-    </row>
-    <row r="128" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N127" s="18"/>
+    </row>
+    <row r="128" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A128" s="4">
         <v>127</v>
       </c>
-      <c r="O128" s="20"/>
-    </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N128" s="20"/>
+    </row>
+    <row r="129" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A129" s="4">
         <v>128</v>
       </c>
-      <c r="O129" s="20"/>
-    </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N129" s="20"/>
+    </row>
+    <row r="130" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A130" s="4">
         <v>129</v>
       </c>
-      <c r="O130" s="20"/>
-    </row>
-    <row r="131" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N130" s="20"/>
+    </row>
+    <row r="131" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A131" s="4">
         <v>130</v>
       </c>
-      <c r="O131" s="20"/>
-    </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N131" s="20"/>
+    </row>
+    <row r="132" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A132" s="4">
         <v>131</v>
       </c>
-      <c r="O132" s="20"/>
-    </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N132" s="20"/>
+    </row>
+    <row r="133" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A133" s="4">
         <v>132</v>
       </c>
-      <c r="O133" s="20"/>
-    </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N133" s="20"/>
+    </row>
+    <row r="134" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A134" s="4">
         <v>133</v>
       </c>
-      <c r="O134" s="20"/>
-    </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N134" s="20"/>
+    </row>
+    <row r="135" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A135" s="4">
         <v>134</v>
       </c>
-      <c r="O135" s="20"/>
-    </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N135" s="20"/>
+    </row>
+    <row r="136" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A136" s="4">
         <v>135</v>
       </c>
-      <c r="O136" s="20"/>
-    </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N136" s="20"/>
+    </row>
+    <row r="137" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A137" s="4">
         <v>136</v>
       </c>
-      <c r="O137" s="20"/>
-    </row>
-    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N137" s="20"/>
+    </row>
+    <row r="138" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A138" s="4">
         <v>137</v>
       </c>
-      <c r="O138" s="20"/>
-    </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N138" s="20"/>
+    </row>
+    <row r="139" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A139" s="4">
         <v>138</v>
       </c>
-      <c r="O139" s="20"/>
-    </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N139" s="20"/>
+    </row>
+    <row r="140" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A140" s="4">
         <v>139</v>
       </c>
-      <c r="O140" s="20"/>
-    </row>
-    <row r="141" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N140" s="20"/>
+    </row>
+    <row r="141" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A141" s="4">
         <v>140</v>
       </c>
-      <c r="O141" s="20"/>
-    </row>
-    <row r="142" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N141" s="20"/>
+    </row>
+    <row r="142" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A142" s="4">
         <v>141</v>
       </c>
-      <c r="O142" s="20"/>
-    </row>
-    <row r="143" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N142" s="20"/>
+    </row>
+    <row r="143" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A143" s="4">
         <v>142</v>
       </c>
-      <c r="O143" s="20"/>
-    </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N143" s="20"/>
+    </row>
+    <row r="144" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A144" s="4">
         <v>143</v>
       </c>
-      <c r="O144" s="20"/>
-    </row>
-    <row r="145" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N144" s="20"/>
+    </row>
+    <row r="145" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A145" s="4">
         <v>144</v>
       </c>
-      <c r="O145" s="20"/>
-    </row>
-    <row r="146" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N145" s="20"/>
+    </row>
+    <row r="146" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A146" s="4">
         <v>145</v>
       </c>
-      <c r="O146" s="20"/>
-    </row>
-    <row r="147" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N146" s="20"/>
+    </row>
+    <row r="147" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A147" s="4">
         <v>146</v>
       </c>
-      <c r="O147" s="20"/>
-    </row>
-    <row r="148" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N147" s="20"/>
+    </row>
+    <row r="148" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A148" s="4">
         <v>147</v>
       </c>
-      <c r="O148" s="20"/>
-    </row>
-    <row r="149" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N148" s="20"/>
+    </row>
+    <row r="149" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A149" s="4">
         <v>148</v>
       </c>
-      <c r="O149" s="20"/>
-    </row>
-    <row r="150" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N149" s="20"/>
+    </row>
+    <row r="150" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A150" s="4">
         <v>149</v>
       </c>
-      <c r="O150" s="20"/>
-    </row>
-    <row r="151" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N150" s="20"/>
+    </row>
+    <row r="151" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A151" s="4">
         <v>150</v>
       </c>
-      <c r="O151" s="20"/>
+      <c r="N151" s="20"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>

</xml_diff>